<commit_message>
feat: biometric fingerprint login, per-question themes, mystery blur, zodiac calculations, and open-ended questions
</commit_message>
<xml_diff>
--- a/Team Building TCKT.xlsx
+++ b/Team Building TCKT.xlsx
@@ -8,25 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NHANDQ\Downloads\TeamBuilding\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9199FD88-83E9-4A76-8F1A-FAB992EB25F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A033379F-AF2E-4A91-B8CF-DED03A245CD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Squizz" sheetId="3" r:id="rId1"/>
-    <sheet name="Bộ Q&amp;A" sheetId="4" r:id="rId2"/>
+    <sheet name="Danh sách tham gia" sheetId="5" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="6" r:id="rId3"/>
+    <sheet name="Bộ Q&amp;A" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId10" roundtripDataChecksum="pgTCipHX9ywkRBr1OQQQksQMWZuIzHSKDim4RXLpGkQ="/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="214">
   <si>
     <t>BỘ 10 CÂU HỎI NHẬP TÊN CHO QUIZIZZ</t>
   </si>
@@ -315,17 +312,381 @@
   <si>
     <t xml:space="preserve">SAU KHI QUÉT QR THAM GIA, TÔI MUỐN HIỆN CÂU HỎI! SAU ĐÓ AE SẼ VIẾT TÊN NGƯỜI ĐÓ LÊN
 -&gt; AI ĐƯỢC NÊU TÊN NHIỀU NHẤT Ở MỖI CÂU HỎI SẼ UỐNG RƯỢU </t>
+  </si>
+  <si>
+    <t>Nguyễn Thị Thùy Dung</t>
+  </si>
+  <si>
+    <t>Nguyễn Thị Hoài Thanh</t>
+  </si>
+  <si>
+    <t>Ngô Thị Nga</t>
+  </si>
+  <si>
+    <t>Đỗ Thị Định</t>
+  </si>
+  <si>
+    <t>Trần Thị Hương</t>
+  </si>
+  <si>
+    <t>Nguyễn Thu Trà</t>
+  </si>
+  <si>
+    <t>Dương Quý Nhân</t>
+  </si>
+  <si>
+    <t>Nguyễn Phương Dung</t>
+  </si>
+  <si>
+    <t>Nguyễn Mai Phương</t>
+  </si>
+  <si>
+    <t>Lã Thị Hồng Vi</t>
+  </si>
+  <si>
+    <t>Trần Thị Đoan Trang</t>
+  </si>
+  <si>
+    <t>Trần Thị Hồng Hạnh</t>
+  </si>
+  <si>
+    <t>Đồng Thị Hồng Ngọc</t>
+  </si>
+  <si>
+    <t>Nguyễn Thuỳ Trang</t>
+  </si>
+  <si>
+    <t>Tô Vũ Châu</t>
+  </si>
+  <si>
+    <t>Phạm Quỳnh Trang</t>
+  </si>
+  <si>
+    <t>Đặng Thanh Hương</t>
+  </si>
+  <si>
+    <t>Đặng Thanh Nhàn</t>
+  </si>
+  <si>
+    <t>Lê Bích An</t>
+  </si>
+  <si>
+    <t>Lê Phương Thảo</t>
+  </si>
+  <si>
+    <t>Nguyễn Thanh Hải</t>
+  </si>
+  <si>
+    <t>Nguyễn Thị Yến</t>
+  </si>
+  <si>
+    <t>Nguyễn Thị Thúy Hằng</t>
+  </si>
+  <si>
+    <t>Nguyễn Minh Hiền</t>
+  </si>
+  <si>
+    <t>Hoàng Huyền Trang</t>
+  </si>
+  <si>
+    <t>Lăng Quốc Toàn</t>
+  </si>
+  <si>
+    <t>Trần Thị Quyên</t>
+  </si>
+  <si>
+    <t>Dương Lan Hương</t>
+  </si>
+  <si>
+    <t>Nguyễn Thị Thu Giang</t>
+  </si>
+  <si>
+    <t>Vũ Lâm Dương</t>
+  </si>
+  <si>
+    <t>Nguyễn Thị Hồng</t>
+  </si>
+  <si>
+    <t>Nguyễn Sông Thương</t>
+  </si>
+  <si>
+    <t>Vũ Thị Mơ</t>
+  </si>
+  <si>
+    <t>Phùng Thu Hường</t>
+  </si>
+  <si>
+    <t>Vương Kim Dung</t>
+  </si>
+  <si>
+    <t>Vũ Lê Anh Thư</t>
+  </si>
+  <si>
+    <t>Đinh Mai Hương</t>
+  </si>
+  <si>
+    <t>Châu Ngọc Anh</t>
+  </si>
+  <si>
+    <t>Nguyễn Ngọc Anh</t>
+  </si>
+  <si>
+    <t>Phạm Thị Thu Hà</t>
+  </si>
+  <si>
+    <t>Trần Đình Lâm</t>
+  </si>
+  <si>
+    <t>Nguyễn Lê Thùy Trang</t>
+  </si>
+  <si>
+    <t>Phạm Thị Hồng Luận</t>
+  </si>
+  <si>
+    <t>Dương Thị Dung</t>
+  </si>
+  <si>
+    <t>Nguyễn Thế Tùng</t>
+  </si>
+  <si>
+    <t>Hồ Quỳnh Trang</t>
+  </si>
+  <si>
+    <t>Đoàn Thị Thương</t>
+  </si>
+  <si>
+    <t>Trưởng phòng</t>
+  </si>
+  <si>
+    <t>Phó phòng</t>
+  </si>
+  <si>
+    <t>KT tiền lương</t>
+  </si>
+  <si>
+    <t>KT thuế</t>
+  </si>
+  <si>
+    <t>Thủ quỹ, KT khoa Cấp cứu</t>
+  </si>
+  <si>
+    <t>KT thanh toán</t>
+  </si>
+  <si>
+    <t>Phân tích dữ liệu</t>
+  </si>
+  <si>
+    <t>KT check doanh số</t>
+  </si>
+  <si>
+    <t>KT ngoại trú</t>
+  </si>
+  <si>
+    <t>KT khoa YHCT, UB</t>
+  </si>
+  <si>
+    <t>KT khoa Nhi, TTSLT</t>
+  </si>
+  <si>
+    <t>KT khoa Nội, GMHS</t>
+  </si>
+  <si>
+    <t>KT khoa Ngoại, TM, KSNK</t>
+  </si>
+  <si>
+    <t>KT khoa LCK, PHCN</t>
+  </si>
+  <si>
+    <t>KT Tài sản</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>KT đoàn khám</t>
+  </si>
+  <si>
+    <t>KTTH</t>
+  </si>
+  <si>
+    <t>KT khoa</t>
+  </si>
+  <si>
+    <t>KT khoa NHM, IVF</t>
+  </si>
+  <si>
+    <t>KT HC khoa Ngoại</t>
+  </si>
+  <si>
+    <t>KT HC khoa Nhi</t>
+  </si>
+  <si>
+    <t>KTHC khoa UB</t>
+  </si>
+  <si>
+    <t>KT nhập liệu</t>
+  </si>
+  <si>
+    <t>XHĐ</t>
+  </si>
+  <si>
+    <t>Leader TN Ngoại trú Tòa A</t>
+  </si>
+  <si>
+    <t>Thu ngân</t>
+  </si>
+  <si>
+    <t>TBP Thu ngân tòa A</t>
+  </si>
+  <si>
+    <t>Leader TN Ngoại trú Tòa D</t>
+  </si>
+  <si>
+    <t>TBP Thu ngân tòa D</t>
+  </si>
+  <si>
+    <t>Học việc</t>
+  </si>
+  <si>
+    <t>Họ và tên</t>
+  </si>
+  <si>
+    <t>Chức vụ</t>
+  </si>
+  <si>
+    <t>STT</t>
+  </si>
+  <si>
+    <t>Mã vân tay</t>
+  </si>
+  <si>
+    <t>Ngày tháng năm sinh</t>
+  </si>
+  <si>
+    <t>13/12/1994</t>
+  </si>
+  <si>
+    <t>13/11/2002</t>
+  </si>
+  <si>
+    <t>19/03/2002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26/06/1992 </t>
+  </si>
+  <si>
+    <t>18/04/2000</t>
+  </si>
+  <si>
+    <t>16/12/2003</t>
+  </si>
+  <si>
+    <t>23/12/1990</t>
+  </si>
+  <si>
+    <t>25/6/1991</t>
+  </si>
+  <si>
+    <t>20/12/1981</t>
+  </si>
+  <si>
+    <t>22/4/1987</t>
+  </si>
+  <si>
+    <t>14/10/2001</t>
+  </si>
+  <si>
+    <t>17/05/1990</t>
+  </si>
+  <si>
+    <t>23/12/1992</t>
+  </si>
+  <si>
+    <t>22/11/1999</t>
+  </si>
+  <si>
+    <t>27/06/2002</t>
+  </si>
+  <si>
+    <t>26/07/2002</t>
+  </si>
+  <si>
+    <t>27/07/2003</t>
+  </si>
+  <si>
+    <t>31/10/2002</t>
+  </si>
+  <si>
+    <t>20/06/2004</t>
+  </si>
+  <si>
+    <t>14/01/1992</t>
+  </si>
+  <si>
+    <t>02/08/1994</t>
+  </si>
+  <si>
+    <t>28/12/2002</t>
+  </si>
+  <si>
+    <t>02/05/2001</t>
+  </si>
+  <si>
+    <t>15/05/1996</t>
+  </si>
+  <si>
+    <t>13/10/2003</t>
+  </si>
+  <si>
+    <t>23/03/2004</t>
+  </si>
+  <si>
+    <t>30/04/1996</t>
+  </si>
+  <si>
+    <t>27/12/1983</t>
+  </si>
+  <si>
+    <t>29/03/2003</t>
+  </si>
+  <si>
+    <t>19/02/2003</t>
+  </si>
+  <si>
+    <t>21/09/2005</t>
+  </si>
+  <si>
+    <t>18/06/2025</t>
+  </si>
+  <si>
+    <t>29/09/2004</t>
+  </si>
+  <si>
+    <t>VIP</t>
+  </si>
+  <si>
+    <t>24/11/2004</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="168" formatCode="dd/mm/yyyy"/>
+  </numFmts>
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -397,6 +758,36 @@
       <family val="2"/>
       <scheme val="major"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -412,7 +803,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -420,47 +811,343 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="14" fontId="11" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="11" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="11" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="11" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="13" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="11" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="11" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="15" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="11" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="11" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="11" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{044B16A6-DC3D-4E23-B159-EFE378109F1C}"/>
+    <cellStyle name="Normal 2 11" xfId="2" xr:uid="{1B00C19F-E8B6-41C6-8FC3-2C8687F210AD}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -679,349 +1366,349 @@
   <dimension ref="A1:L81"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="14.42578125" style="14"/>
+    <col min="1" max="16384" width="14.42578125" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="144" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="J1" s="15"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="J1" s="9"/>
     </row>
     <row r="2" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="10" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="11" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="18"/>
+      <c r="A4" s="12"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="13" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="20"/>
+      <c r="A6" s="14"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="13" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="20"/>
+      <c r="A8" s="14"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="L9" s="14" t="s">
+      <c r="L9" s="8" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A10" s="17"/>
+      <c r="A10" s="11"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="11" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="18"/>
+      <c r="A12" s="12"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="13" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="20"/>
+      <c r="A14" s="14"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="13" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="20"/>
+      <c r="A16" s="14"/>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="19" t="s">
+      <c r="A17" s="13" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="17"/>
+      <c r="A18" s="11"/>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="17" t="s">
+      <c r="A19" s="11" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="18"/>
+      <c r="A20" s="12"/>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" s="19" t="s">
+      <c r="A21" s="13" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="20"/>
+      <c r="A22" s="14"/>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" s="19" t="s">
+      <c r="A23" s="13" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="24" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="20"/>
+      <c r="A24" s="14"/>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" s="19" t="s">
+      <c r="A25" s="13" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" s="17"/>
+      <c r="A26" s="11"/>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" s="17" t="s">
+      <c r="A27" s="11" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="28" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="18"/>
+      <c r="A28" s="12"/>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" s="19" t="s">
+      <c r="A29" s="13" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="30" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="20"/>
+      <c r="A30" s="14"/>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A31" s="19" t="s">
+      <c r="A31" s="13" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="32" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A32" s="20"/>
+      <c r="A32" s="14"/>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" s="19" t="s">
+      <c r="A33" s="13" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" s="17"/>
+      <c r="A34" s="11"/>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35" s="17" t="s">
+      <c r="A35" s="11" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="36" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A36" s="18"/>
+      <c r="A36" s="12"/>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A37" s="19" t="s">
+      <c r="A37" s="13" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="38" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A38" s="20"/>
+      <c r="A38" s="14"/>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A39" s="19" t="s">
+      <c r="A39" s="13" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="40" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A40" s="20"/>
+      <c r="A40" s="14"/>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A41" s="19" t="s">
+      <c r="A41" s="13" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A42" s="17"/>
+      <c r="A42" s="11"/>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A43" s="17" t="s">
+      <c r="A43" s="11" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="44" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A44" s="18"/>
+      <c r="A44" s="12"/>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A45" s="19" t="s">
+      <c r="A45" s="13" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="46" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A46" s="20"/>
+      <c r="A46" s="14"/>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A47" s="19" t="s">
+      <c r="A47" s="13" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="48" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A48" s="20"/>
+      <c r="A48" s="14"/>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A49" s="19" t="s">
+      <c r="A49" s="13" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A50" s="17"/>
+      <c r="A50" s="11"/>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A51" s="17" t="s">
+      <c r="A51" s="11" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="52" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A52" s="18"/>
+      <c r="A52" s="12"/>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A53" s="19" t="s">
+      <c r="A53" s="13" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="54" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A54" s="20"/>
+      <c r="A54" s="14"/>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A55" s="19" t="s">
+      <c r="A55" s="13" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="56" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A56" s="20"/>
+      <c r="A56" s="14"/>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A57" s="19" t="s">
+      <c r="A57" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="K57" s="14" t="s">
+      <c r="K57" s="8" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A58" s="17"/>
+      <c r="A58" s="11"/>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A59" s="17" t="s">
+      <c r="A59" s="11" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="60" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A60" s="18"/>
+      <c r="A60" s="12"/>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A61" s="19" t="s">
+      <c r="A61" s="13" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="62" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A62" s="20"/>
+      <c r="A62" s="14"/>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A63" s="19" t="s">
+      <c r="A63" s="13" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="64" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A64" s="20"/>
+      <c r="A64" s="14"/>
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A65" s="19" t="s">
+      <c r="A65" s="13" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A66" s="17"/>
+      <c r="A66" s="11"/>
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A67" s="17" t="s">
+      <c r="A67" s="11" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="68" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A68" s="18"/>
+      <c r="A68" s="12"/>
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A69" s="19" t="s">
+      <c r="A69" s="13" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="70" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A70" s="20"/>
+      <c r="A70" s="14"/>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A71" s="19" t="s">
+      <c r="A71" s="13" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="72" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A72" s="20"/>
+      <c r="A72" s="14"/>
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A73" s="19" t="s">
+      <c r="A73" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="L73" s="14" t="s">
+      <c r="L73" s="8" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A74" s="17"/>
+      <c r="A74" s="11"/>
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A75" s="17" t="s">
+      <c r="A75" s="11" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="76" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A76" s="18"/>
+      <c r="A76" s="12"/>
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A77" s="19" t="s">
+      <c r="A77" s="13" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="78" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A78" s="20"/>
+      <c r="A78" s="14"/>
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A79" s="19" t="s">
+      <c r="A79" s="13" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="80" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A80" s="20"/>
+      <c r="A80" s="14"/>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A81" s="19" t="s">
+      <c r="A81" s="13" t="s">
         <v>59</v>
       </c>
     </row>
@@ -1034,6 +1721,1849 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E75B50C-99D4-4954-9C5A-E9372A08BF64}">
+  <dimension ref="A1:E48"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="5.5703125" customWidth="1"/>
+    <col min="2" max="2" width="23" style="29" customWidth="1"/>
+    <col min="3" max="3" width="25.7109375" customWidth="1"/>
+    <col min="4" max="4" width="16.42578125" customWidth="1"/>
+    <col min="5" max="5" width="26.140625" style="55" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="23" t="s">
+        <v>176</v>
+      </c>
+      <c r="B1" s="26" t="s">
+        <v>174</v>
+      </c>
+      <c r="C1" s="26" t="s">
+        <v>175</v>
+      </c>
+      <c r="D1" s="22" t="s">
+        <v>177</v>
+      </c>
+      <c r="E1" s="54" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="24">
+        <v>1</v>
+      </c>
+      <c r="B2" s="27" t="s">
+        <v>96</v>
+      </c>
+      <c r="C2" s="27" t="s">
+        <v>143</v>
+      </c>
+      <c r="D2" s="24">
+        <v>6</v>
+      </c>
+      <c r="E2" s="55">
+        <v>33873</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="25">
+        <v>2</v>
+      </c>
+      <c r="B3" s="27" t="s">
+        <v>97</v>
+      </c>
+      <c r="C3" s="27" t="s">
+        <v>144</v>
+      </c>
+      <c r="D3" s="25">
+        <v>1770</v>
+      </c>
+      <c r="E3" s="55">
+        <v>33438</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="25">
+        <v>3</v>
+      </c>
+      <c r="B4" s="27" t="s">
+        <v>98</v>
+      </c>
+      <c r="C4" s="27" t="s">
+        <v>145</v>
+      </c>
+      <c r="D4" s="25">
+        <v>8</v>
+      </c>
+      <c r="E4" s="55">
+        <v>34857</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="25">
+        <v>4</v>
+      </c>
+      <c r="B5" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="C5" s="27" t="s">
+        <v>146</v>
+      </c>
+      <c r="D5" s="25">
+        <v>2539</v>
+      </c>
+      <c r="E5" s="55">
+        <v>32742</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="25">
+        <v>5</v>
+      </c>
+      <c r="B6" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="C6" s="27" t="s">
+        <v>147</v>
+      </c>
+      <c r="D6" s="25">
+        <v>381</v>
+      </c>
+      <c r="E6" s="55">
+        <v>35183</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="25">
+        <v>6</v>
+      </c>
+      <c r="B7" s="27" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7" s="27" t="s">
+        <v>148</v>
+      </c>
+      <c r="D7" s="25">
+        <v>3765</v>
+      </c>
+      <c r="E7" s="55">
+        <v>33775</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="25">
+        <v>7</v>
+      </c>
+      <c r="B8" s="27" t="s">
+        <v>102</v>
+      </c>
+      <c r="C8" s="27" t="s">
+        <v>149</v>
+      </c>
+      <c r="D8" s="25">
+        <v>2310</v>
+      </c>
+      <c r="E8" s="54">
+        <v>34681</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="25">
+        <v>8</v>
+      </c>
+      <c r="B9" s="27" t="s">
+        <v>103</v>
+      </c>
+      <c r="C9" s="27" t="s">
+        <v>150</v>
+      </c>
+      <c r="D9" s="25">
+        <v>3761</v>
+      </c>
+      <c r="E9" s="55">
+        <v>36483</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="25">
+        <v>9</v>
+      </c>
+      <c r="B10" s="27" t="s">
+        <v>104</v>
+      </c>
+      <c r="C10" s="27" t="s">
+        <v>151</v>
+      </c>
+      <c r="D10" s="25">
+        <v>1437</v>
+      </c>
+      <c r="E10" s="55">
+        <v>36122</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="25">
+        <v>10</v>
+      </c>
+      <c r="B11" s="27" t="s">
+        <v>105</v>
+      </c>
+      <c r="C11" s="27" t="s">
+        <v>152</v>
+      </c>
+      <c r="D11" s="25">
+        <v>1717</v>
+      </c>
+      <c r="E11" s="55">
+        <v>36171</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="25">
+        <v>11</v>
+      </c>
+      <c r="B12" s="27" t="s">
+        <v>106</v>
+      </c>
+      <c r="C12" s="27" t="s">
+        <v>153</v>
+      </c>
+      <c r="D12" s="25">
+        <v>2462</v>
+      </c>
+      <c r="E12" s="55">
+        <v>34230</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="25">
+        <v>12</v>
+      </c>
+      <c r="B13" s="27" t="s">
+        <v>107</v>
+      </c>
+      <c r="C13" s="27" t="s">
+        <v>154</v>
+      </c>
+      <c r="D13" s="25">
+        <v>2836</v>
+      </c>
+      <c r="E13" s="55">
+        <v>37046</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="25">
+        <v>13</v>
+      </c>
+      <c r="B14" s="27" t="s">
+        <v>108</v>
+      </c>
+      <c r="C14" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="D14" s="25">
+        <v>3398</v>
+      </c>
+      <c r="E14" s="55">
+        <v>35769</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="25">
+        <v>14</v>
+      </c>
+      <c r="B15" s="27" t="s">
+        <v>109</v>
+      </c>
+      <c r="C15" s="27" t="s">
+        <v>156</v>
+      </c>
+      <c r="D15" s="25">
+        <v>4210</v>
+      </c>
+      <c r="E15" s="55">
+        <v>37723</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="25">
+        <v>15</v>
+      </c>
+      <c r="B16" s="27" t="s">
+        <v>110</v>
+      </c>
+      <c r="C16" s="27" t="s">
+        <v>157</v>
+      </c>
+      <c r="D16" s="25">
+        <v>4339</v>
+      </c>
+      <c r="E16" s="55">
+        <v>35675</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="25">
+        <v>16</v>
+      </c>
+      <c r="B17" s="27" t="s">
+        <v>111</v>
+      </c>
+      <c r="C17" s="27" t="s">
+        <v>158</v>
+      </c>
+      <c r="D17" s="25">
+        <v>4151</v>
+      </c>
+      <c r="E17" s="55">
+        <v>37334</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="25">
+        <v>17</v>
+      </c>
+      <c r="B18" s="27" t="s">
+        <v>112</v>
+      </c>
+      <c r="C18" s="27" t="s">
+        <v>159</v>
+      </c>
+      <c r="D18" s="25">
+        <v>5117</v>
+      </c>
+      <c r="E18" s="55">
+        <v>37324</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="25">
+        <v>18</v>
+      </c>
+      <c r="B19" s="27" t="s">
+        <v>113</v>
+      </c>
+      <c r="C19" s="27" t="s">
+        <v>160</v>
+      </c>
+      <c r="D19" s="25">
+        <v>5679</v>
+      </c>
+      <c r="E19" s="55">
+        <v>33781</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="25">
+        <v>19</v>
+      </c>
+      <c r="B20" s="27" t="s">
+        <v>114</v>
+      </c>
+      <c r="C20" s="27" t="s">
+        <v>161</v>
+      </c>
+      <c r="D20" s="25">
+        <v>5788</v>
+      </c>
+      <c r="E20" s="55">
+        <v>38025</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="25">
+        <v>20</v>
+      </c>
+      <c r="B21" s="27" t="s">
+        <v>115</v>
+      </c>
+      <c r="C21" s="27" t="s">
+        <v>161</v>
+      </c>
+      <c r="D21" s="25">
+        <v>5823</v>
+      </c>
+      <c r="E21" s="55">
+        <v>36903</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="25">
+        <v>21</v>
+      </c>
+      <c r="B22" s="27" t="s">
+        <v>116</v>
+      </c>
+      <c r="C22" s="27" t="s">
+        <v>162</v>
+      </c>
+      <c r="D22" s="25">
+        <v>3159</v>
+      </c>
+      <c r="E22" s="55">
+        <v>34548</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="25">
+        <v>22</v>
+      </c>
+      <c r="B23" s="27" t="s">
+        <v>117</v>
+      </c>
+      <c r="C23" s="27" t="s">
+        <v>163</v>
+      </c>
+      <c r="D23" s="25">
+        <v>3628</v>
+      </c>
+      <c r="E23" s="55">
+        <v>36565</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="25">
+        <v>23</v>
+      </c>
+      <c r="B24" s="27" t="s">
+        <v>118</v>
+      </c>
+      <c r="C24" s="27" t="s">
+        <v>164</v>
+      </c>
+      <c r="D24" s="25">
+        <v>4257</v>
+      </c>
+      <c r="E24" s="55">
+        <v>33010</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="25">
+        <v>24</v>
+      </c>
+      <c r="B25" s="27" t="s">
+        <v>119</v>
+      </c>
+      <c r="C25" s="27" t="s">
+        <v>165</v>
+      </c>
+      <c r="D25" s="25">
+        <v>6040</v>
+      </c>
+      <c r="E25" s="55">
+        <v>36486</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="25">
+        <v>25</v>
+      </c>
+      <c r="B26" s="27" t="s">
+        <v>120</v>
+      </c>
+      <c r="C26" s="27" t="s">
+        <v>166</v>
+      </c>
+      <c r="D26" s="25">
+        <v>4049</v>
+      </c>
+      <c r="E26" s="55">
+        <v>37434</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="25">
+        <v>26</v>
+      </c>
+      <c r="B27" s="27" t="s">
+        <v>121</v>
+      </c>
+      <c r="C27" s="27" t="s">
+        <v>166</v>
+      </c>
+      <c r="D27" s="25">
+        <v>4048</v>
+      </c>
+      <c r="E27" s="55">
+        <v>37463</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="25">
+        <v>27</v>
+      </c>
+      <c r="B28" s="27" t="s">
+        <v>122</v>
+      </c>
+      <c r="C28" s="27" t="s">
+        <v>166</v>
+      </c>
+      <c r="D28" s="25">
+        <v>4330</v>
+      </c>
+      <c r="E28" s="55">
+        <v>37829</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="25">
+        <v>28</v>
+      </c>
+      <c r="B29" s="27" t="s">
+        <v>123</v>
+      </c>
+      <c r="C29" s="27" t="s">
+        <v>166</v>
+      </c>
+      <c r="D29" s="25">
+        <v>4340</v>
+      </c>
+      <c r="E29" s="55">
+        <v>37560</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="25">
+        <v>29</v>
+      </c>
+      <c r="B30" s="27" t="s">
+        <v>124</v>
+      </c>
+      <c r="C30" s="27" t="s">
+        <v>166</v>
+      </c>
+      <c r="D30" s="25">
+        <v>4391</v>
+      </c>
+      <c r="E30" s="55">
+        <v>37927</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="25">
+        <v>30</v>
+      </c>
+      <c r="B31" s="27" t="s">
+        <v>125</v>
+      </c>
+      <c r="C31" s="27" t="s">
+        <v>166</v>
+      </c>
+      <c r="D31" s="25">
+        <v>5381</v>
+      </c>
+      <c r="E31" s="55">
+        <v>38158</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="25">
+        <v>31</v>
+      </c>
+      <c r="B32" s="27" t="s">
+        <v>126</v>
+      </c>
+      <c r="C32" s="27" t="s">
+        <v>166</v>
+      </c>
+      <c r="D32" s="25">
+        <v>5821</v>
+      </c>
+      <c r="E32" s="55">
+        <v>38330</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="25">
+        <v>32</v>
+      </c>
+      <c r="B33" s="27" t="s">
+        <v>127</v>
+      </c>
+      <c r="C33" s="27" t="s">
+        <v>166</v>
+      </c>
+      <c r="D33" s="25">
+        <v>6038</v>
+      </c>
+      <c r="E33" s="54">
+        <v>37983</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="25">
+        <v>33</v>
+      </c>
+      <c r="B34" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="C34" s="27" t="s">
+        <v>167</v>
+      </c>
+      <c r="D34" s="25">
+        <v>2503</v>
+      </c>
+      <c r="E34" s="55">
+        <v>33617</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="25">
+        <v>34</v>
+      </c>
+      <c r="B35" s="27" t="s">
+        <v>129</v>
+      </c>
+      <c r="C35" s="27" t="s">
+        <v>167</v>
+      </c>
+      <c r="D35" s="25">
+        <v>4159</v>
+      </c>
+      <c r="E35" s="55">
+        <v>37013</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="25">
+        <v>35</v>
+      </c>
+      <c r="B36" s="27" t="s">
+        <v>130</v>
+      </c>
+      <c r="C36" s="27" t="s">
+        <v>167</v>
+      </c>
+      <c r="D36" s="25">
+        <v>4404</v>
+      </c>
+      <c r="E36" s="55">
+        <v>35200</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="25">
+        <v>36</v>
+      </c>
+      <c r="B37" s="27" t="s">
+        <v>131</v>
+      </c>
+      <c r="C37" s="27" t="s">
+        <v>167</v>
+      </c>
+      <c r="D37" s="25">
+        <v>4846</v>
+      </c>
+      <c r="E37" s="55">
+        <v>37907</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="25">
+        <v>37</v>
+      </c>
+      <c r="B38" s="27" t="s">
+        <v>132</v>
+      </c>
+      <c r="C38" s="27" t="s">
+        <v>168</v>
+      </c>
+      <c r="D38" s="25">
+        <v>2971</v>
+      </c>
+      <c r="E38" s="55">
+        <v>36490</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="25">
+        <v>38</v>
+      </c>
+      <c r="B39" s="27" t="s">
+        <v>133</v>
+      </c>
+      <c r="C39" s="27" t="s">
+        <v>169</v>
+      </c>
+      <c r="D39" s="25">
+        <v>2877</v>
+      </c>
+      <c r="E39" s="55">
+        <v>36903</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="25">
+        <v>39</v>
+      </c>
+      <c r="B40" s="27" t="s">
+        <v>134</v>
+      </c>
+      <c r="C40" s="27" t="s">
+        <v>169</v>
+      </c>
+      <c r="D40" s="25">
+        <v>4565</v>
+      </c>
+      <c r="E40" s="55">
+        <v>33516</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="25">
+        <v>40</v>
+      </c>
+      <c r="B41" s="27" t="s">
+        <v>135</v>
+      </c>
+      <c r="C41" s="27" t="s">
+        <v>170</v>
+      </c>
+      <c r="D41" s="25">
+        <v>886</v>
+      </c>
+      <c r="E41" s="55">
+        <v>34777</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="25">
+        <v>41</v>
+      </c>
+      <c r="B42" s="27" t="s">
+        <v>136</v>
+      </c>
+      <c r="C42" s="27" t="s">
+        <v>169</v>
+      </c>
+      <c r="D42" s="25">
+        <v>3958</v>
+      </c>
+      <c r="E42" s="55">
+        <v>37505</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="25">
+        <v>42</v>
+      </c>
+      <c r="B43" s="27" t="s">
+        <v>137</v>
+      </c>
+      <c r="C43" s="27" t="s">
+        <v>169</v>
+      </c>
+      <c r="D43" s="25">
+        <v>2144</v>
+      </c>
+      <c r="E43" s="55">
+        <v>36938</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="25">
+        <v>43</v>
+      </c>
+      <c r="B44" s="27" t="s">
+        <v>138</v>
+      </c>
+      <c r="C44" s="27" t="s">
+        <v>171</v>
+      </c>
+      <c r="D44" s="25">
+        <v>3379</v>
+      </c>
+      <c r="E44" s="55">
+        <v>34462</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="25">
+        <v>44</v>
+      </c>
+      <c r="B45" s="27" t="s">
+        <v>139</v>
+      </c>
+      <c r="C45" s="27" t="s">
+        <v>172</v>
+      </c>
+      <c r="D45" s="25">
+        <v>2200</v>
+      </c>
+      <c r="E45" s="55">
+        <v>33414</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="25">
+        <v>45</v>
+      </c>
+      <c r="B46" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="C46" s="28" t="s">
+        <v>212</v>
+      </c>
+      <c r="D46" s="21">
+        <v>641</v>
+      </c>
+      <c r="E46" s="55" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="25">
+        <v>46</v>
+      </c>
+      <c r="B47" s="27" t="s">
+        <v>141</v>
+      </c>
+      <c r="C47" s="27" t="s">
+        <v>173</v>
+      </c>
+      <c r="D47" s="25">
+        <v>6248</v>
+      </c>
+      <c r="E47" s="54" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="25">
+        <v>47</v>
+      </c>
+      <c r="B48" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="C48" s="27" t="s">
+        <v>169</v>
+      </c>
+      <c r="D48" s="25">
+        <v>5791</v>
+      </c>
+      <c r="E48" s="54">
+        <v>38160</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4846012-1C8E-45A4-8F94-FFA376830FDA}">
+  <dimension ref="A1:B131"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.42578125" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A1" s="31" t="s">
+        <v>177</v>
+      </c>
+      <c r="B1" s="47" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="33">
+        <v>6</v>
+      </c>
+      <c r="B2" s="48">
+        <v>33873</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="36">
+        <v>1770</v>
+      </c>
+      <c r="B3" s="49">
+        <v>33438</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="35">
+        <v>8</v>
+      </c>
+      <c r="B4" s="49">
+        <v>34886</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="37">
+        <v>2539</v>
+      </c>
+      <c r="B5" s="49">
+        <v>32742</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="36">
+        <v>381</v>
+      </c>
+      <c r="B6" s="49">
+        <v>35183</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="37">
+        <v>3765</v>
+      </c>
+      <c r="B7" s="49">
+        <v>33775</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="37">
+        <v>2310</v>
+      </c>
+      <c r="B8" s="49" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="37">
+        <v>3761</v>
+      </c>
+      <c r="B9" s="49">
+        <v>36483</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="36">
+        <v>1236</v>
+      </c>
+      <c r="B10" s="49">
+        <v>33332</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="36">
+        <v>1437</v>
+      </c>
+      <c r="B11" s="49">
+        <v>36122</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="35">
+        <v>1717</v>
+      </c>
+      <c r="B12" s="49">
+        <v>36465</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="37">
+        <v>2462</v>
+      </c>
+      <c r="B13" s="49">
+        <v>34230</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="36">
+        <v>2836</v>
+      </c>
+      <c r="B14" s="49">
+        <v>36987</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="35">
+        <v>3398</v>
+      </c>
+      <c r="B15" s="49">
+        <v>35562</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="37">
+        <v>4210</v>
+      </c>
+      <c r="B16" s="49">
+        <v>37959</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="37">
+        <v>4663</v>
+      </c>
+      <c r="B17" s="49" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="37">
+        <v>4339</v>
+      </c>
+      <c r="B18" s="49">
+        <v>35470</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="37">
+        <v>4151</v>
+      </c>
+      <c r="B19" s="49" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A20" s="37">
+        <v>5117</v>
+      </c>
+      <c r="B20" s="49">
+        <v>37502</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="37">
+        <v>5679</v>
+      </c>
+      <c r="B21" s="49" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="37">
+        <v>5426</v>
+      </c>
+      <c r="B22" s="49" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="37">
+        <v>5747</v>
+      </c>
+      <c r="B23" s="49" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A24" s="37">
+        <v>5788</v>
+      </c>
+      <c r="B24" s="49">
+        <v>38201</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="37">
+        <v>5823</v>
+      </c>
+      <c r="B25" s="49">
+        <v>37226</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A26" s="32"/>
+      <c r="B26" s="50"/>
+    </row>
+    <row r="27" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A27" s="38">
+        <v>1862</v>
+      </c>
+      <c r="B27" s="44" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A28" s="36">
+        <v>2973</v>
+      </c>
+      <c r="B28" s="43" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A29" s="37">
+        <v>3326</v>
+      </c>
+      <c r="B29" s="43">
+        <v>31626</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A30" s="37">
+        <v>3268</v>
+      </c>
+      <c r="B30" s="43" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A31" s="37">
+        <v>4013</v>
+      </c>
+      <c r="B31" s="43" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A32" s="37">
+        <v>3306</v>
+      </c>
+      <c r="B32" s="43" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A33" s="37">
+        <v>3628</v>
+      </c>
+      <c r="B33" s="43">
+        <v>36771</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A34" s="37">
+        <v>4257</v>
+      </c>
+      <c r="B34" s="43" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A35" s="37">
+        <v>5789</v>
+      </c>
+      <c r="B35" s="43">
+        <v>30691</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A36" s="37">
+        <v>5328</v>
+      </c>
+      <c r="B36" s="43" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A37" s="38">
+        <v>6040</v>
+      </c>
+      <c r="B37" s="51" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A38" s="32"/>
+      <c r="B38" s="50"/>
+    </row>
+    <row r="39" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A39" s="37">
+        <v>4049</v>
+      </c>
+      <c r="B39" s="45" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A40" s="37">
+        <v>4048</v>
+      </c>
+      <c r="B40" s="43" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A41" s="37">
+        <v>4047</v>
+      </c>
+      <c r="B41" s="43">
+        <v>37961</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A42" s="37">
+        <v>4330</v>
+      </c>
+      <c r="B42" s="43" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A43" s="37">
+        <v>4340</v>
+      </c>
+      <c r="B43" s="43" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A44" s="37">
+        <v>4391</v>
+      </c>
+      <c r="B44" s="43">
+        <v>37663</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A45" s="37">
+        <v>5381</v>
+      </c>
+      <c r="B45" s="43" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A46" s="37">
+        <v>5675</v>
+      </c>
+      <c r="B46" s="43">
+        <v>36536</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A47" s="37">
+        <v>5821</v>
+      </c>
+      <c r="B47" s="43">
+        <v>38242</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" s="30"/>
+      <c r="B48" s="42"/>
+    </row>
+    <row r="49" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A49" s="37"/>
+      <c r="B49" s="49"/>
+    </row>
+    <row r="50" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A50" s="37"/>
+      <c r="B50" s="49"/>
+    </row>
+    <row r="51" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A51" s="40"/>
+      <c r="B51" s="50"/>
+    </row>
+    <row r="52" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A52" s="34">
+        <v>2503</v>
+      </c>
+      <c r="B52" s="52" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A53" s="37">
+        <v>3159</v>
+      </c>
+      <c r="B53" s="52" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A54" s="37">
+        <v>3269</v>
+      </c>
+      <c r="B54" s="49" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A55" s="37">
+        <v>4159</v>
+      </c>
+      <c r="B55" s="52" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A56" s="37">
+        <v>4404</v>
+      </c>
+      <c r="B56" s="52" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A57" s="37">
+        <v>4846</v>
+      </c>
+      <c r="B57" s="52" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A58" s="37">
+        <v>6014</v>
+      </c>
+      <c r="B58" s="52" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A59" s="37"/>
+      <c r="B59" s="52"/>
+    </row>
+    <row r="60" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A60" s="37"/>
+      <c r="B60" s="52"/>
+    </row>
+    <row r="61" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A61" s="37"/>
+      <c r="B61" s="52"/>
+    </row>
+    <row r="62" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A62" s="40"/>
+      <c r="B62" s="50"/>
+    </row>
+    <row r="63" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A63" s="33">
+        <v>1790</v>
+      </c>
+      <c r="B63" s="48">
+        <v>31292</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A64" s="36">
+        <v>2077</v>
+      </c>
+      <c r="B64" s="49">
+        <v>36652</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A65" s="37">
+        <v>2200</v>
+      </c>
+      <c r="B65" s="49">
+        <v>33414</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A66" s="35">
+        <v>2209</v>
+      </c>
+      <c r="B66" s="49">
+        <v>30572</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A67" s="36">
+        <v>2560</v>
+      </c>
+      <c r="B67" s="49">
+        <v>37033</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A68" s="35">
+        <v>2569</v>
+      </c>
+      <c r="B68" s="49">
+        <v>36919</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A69" s="36">
+        <v>2622</v>
+      </c>
+      <c r="B69" s="49">
+        <v>37108</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A70" s="36">
+        <v>2680</v>
+      </c>
+      <c r="B70" s="49">
+        <v>37178</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A71" s="36">
+        <v>2805</v>
+      </c>
+      <c r="B71" s="49">
+        <v>36541</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A72" s="36">
+        <v>3041</v>
+      </c>
+      <c r="B72" s="49">
+        <v>35692</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A73" s="37">
+        <v>2668</v>
+      </c>
+      <c r="B73" s="49">
+        <v>35202</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A74" s="35">
+        <v>1811</v>
+      </c>
+      <c r="B74" s="49">
+        <v>35395</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A75" s="37">
+        <v>2143</v>
+      </c>
+      <c r="B75" s="49">
+        <v>36018</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A76" s="35">
+        <v>886</v>
+      </c>
+      <c r="B76" s="49">
+        <v>34777</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A77" s="35">
+        <v>2563</v>
+      </c>
+      <c r="B77" s="49">
+        <v>36264</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A78" s="35">
+        <v>2293</v>
+      </c>
+      <c r="B78" s="49">
+        <v>34924</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A79" s="35">
+        <v>2494</v>
+      </c>
+      <c r="B79" s="49">
+        <v>36174</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A80" s="35">
+        <v>2971</v>
+      </c>
+      <c r="B80" s="49">
+        <v>36490</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A81" s="35">
+        <v>2877</v>
+      </c>
+      <c r="B81" s="49">
+        <v>37226</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A82" s="35">
+        <v>3363</v>
+      </c>
+      <c r="B82" s="49">
+        <v>36854</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A83" s="35">
+        <v>3426</v>
+      </c>
+      <c r="B83" s="49">
+        <v>37569</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A84" s="35">
+        <v>3476</v>
+      </c>
+      <c r="B84" s="49">
+        <v>36571</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A85" s="35">
+        <v>3474</v>
+      </c>
+      <c r="B85" s="49">
+        <v>36950</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A86" s="35">
+        <v>3379</v>
+      </c>
+      <c r="B86" s="49">
+        <v>34551</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A87" s="35">
+        <v>670</v>
+      </c>
+      <c r="B87" s="49"/>
+    </row>
+    <row r="88" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A88" s="35">
+        <v>850</v>
+      </c>
+      <c r="B88" s="49">
+        <v>30187</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A89" s="35">
+        <v>2144</v>
+      </c>
+      <c r="B89" s="49">
+        <v>36938</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A90" s="39">
+        <v>3958</v>
+      </c>
+      <c r="B90" s="49">
+        <v>37416</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A91" s="32"/>
+      <c r="B91" s="50"/>
+    </row>
+    <row r="92" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A92" s="35">
+        <v>1779</v>
+      </c>
+      <c r="B92" s="49">
+        <v>29064</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A93" s="32"/>
+      <c r="B93" s="50"/>
+    </row>
+    <row r="94" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A94" s="41">
+        <v>1179</v>
+      </c>
+      <c r="B94" s="49">
+        <v>32435</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A95" s="35">
+        <v>252</v>
+      </c>
+      <c r="B95" s="49">
+        <v>32396</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A96" s="35">
+        <v>3648</v>
+      </c>
+      <c r="B96" s="49">
+        <v>32642</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A97" s="35">
+        <v>3681</v>
+      </c>
+      <c r="B97" s="52">
+        <v>33311</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A98" s="35">
+        <v>3535</v>
+      </c>
+      <c r="B98" s="49">
+        <v>34101</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A99" s="36">
+        <v>1124</v>
+      </c>
+      <c r="B99" s="49">
+        <v>33345</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A100" s="37">
+        <v>3488</v>
+      </c>
+      <c r="B100" s="49">
+        <v>34357</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A101" s="35">
+        <v>2054</v>
+      </c>
+      <c r="B101" s="49"/>
+    </row>
+    <row r="102" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A102" s="37">
+        <v>3946</v>
+      </c>
+      <c r="B102" s="49">
+        <v>36996</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A103" s="37">
+        <v>3943</v>
+      </c>
+      <c r="B103" s="49">
+        <v>37322</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A104" s="37">
+        <v>3936</v>
+      </c>
+      <c r="B104" s="49">
+        <v>37032</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A105" s="37">
+        <v>3937</v>
+      </c>
+      <c r="B105" s="49">
+        <v>36164</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A106" s="37">
+        <v>2954</v>
+      </c>
+      <c r="B106" s="49">
+        <v>34138</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A107" s="37">
+        <v>3588</v>
+      </c>
+      <c r="B107" s="49">
+        <v>36638</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A108" s="37">
+        <v>4182</v>
+      </c>
+      <c r="B108" s="49">
+        <v>37322</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A109" s="37">
+        <v>3511</v>
+      </c>
+      <c r="B109" s="49">
+        <v>35386</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A110" s="37">
+        <v>3870</v>
+      </c>
+      <c r="B110" s="49">
+        <v>36912</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A111" s="37">
+        <v>4186</v>
+      </c>
+      <c r="B111" s="49">
+        <v>35491</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A112" s="37">
+        <v>4502</v>
+      </c>
+      <c r="B112" s="49" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A113" s="37">
+        <v>4495</v>
+      </c>
+      <c r="B113" s="49" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A114" s="37">
+        <v>3910</v>
+      </c>
+      <c r="B114" s="49">
+        <v>35424</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A115" s="37">
+        <v>4352</v>
+      </c>
+      <c r="B115" s="49">
+        <v>37349</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A116" s="37">
+        <v>2638</v>
+      </c>
+      <c r="B116" s="53">
+        <v>33989</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A117" s="37">
+        <v>4888</v>
+      </c>
+      <c r="B117" s="49">
+        <v>36590</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A118" s="37">
+        <v>4320</v>
+      </c>
+      <c r="B118" s="49">
+        <v>37838</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A119" s="37">
+        <v>4887</v>
+      </c>
+      <c r="B119" s="49">
+        <v>37804</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A120" s="37">
+        <v>4422</v>
+      </c>
+      <c r="B120" s="49">
+        <v>37692</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A121" s="37">
+        <v>4296</v>
+      </c>
+      <c r="B121" s="49" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A122" s="37">
+        <v>4351</v>
+      </c>
+      <c r="B122" s="49">
+        <v>37690</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A123" s="37">
+        <v>4295</v>
+      </c>
+      <c r="B123" s="49" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A124" s="37">
+        <v>5229</v>
+      </c>
+      <c r="B124" s="49">
+        <v>32662</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A125" s="37">
+        <v>5170</v>
+      </c>
+      <c r="B125" s="49">
+        <v>37149</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A126" s="37">
+        <v>4782</v>
+      </c>
+      <c r="B126" s="49" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A127" s="37">
+        <v>4680</v>
+      </c>
+      <c r="B127" s="49" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A128" s="37">
+        <v>5742</v>
+      </c>
+      <c r="B128" s="49">
+        <v>37811</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A129" s="37">
+        <v>4358</v>
+      </c>
+      <c r="B129" s="49">
+        <v>37662</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A130" s="37">
+        <v>5632</v>
+      </c>
+      <c r="B130" s="52">
+        <v>36258</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A131" s="37">
+        <v>5631</v>
+      </c>
+      <c r="B131" s="46" t="s">
+        <v>211</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -1045,10 +3575,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="8"/>
+      <c r="B1" s="18"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -1059,27 +3589,27 @@
       <c r="J1" s="1"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="C3" s="8"/>
+      <c r="C3" s="18"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -1137,28 +3667,28 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
+      <c r="B7" s="18"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="18"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
@@ -1170,11 +3700,11 @@
       <c r="A9" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="18"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
@@ -1202,11 +3732,11 @@
       <c r="A11" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
@@ -1303,8 +3833,8 @@
       <c r="A18" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B18" s="9"/>
-      <c r="C18" s="8"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="18"/>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
@@ -1332,8 +3862,8 @@
       <c r="A20" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B20" s="9"/>
-      <c r="C20" s="8"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="18"/>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
@@ -1346,8 +3876,8 @@
       <c r="A21" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="B21" s="9"/>
-      <c r="C21" s="8"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="18"/>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
@@ -1375,8 +3905,8 @@
       <c r="A23" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="B23" s="11"/>
-      <c r="C23" s="8"/>
+      <c r="B23" s="20"/>
+      <c r="C23" s="18"/>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
@@ -1389,8 +3919,8 @@
       <c r="A24" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="B24" s="9"/>
-      <c r="C24" s="8"/>
+      <c r="B24" s="17"/>
+      <c r="C24" s="18"/>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
@@ -1402,8 +3932,8 @@
       <c r="A25" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B25" s="9"/>
-      <c r="C25" s="8"/>
+      <c r="B25" s="17"/>
+      <c r="C25" s="18"/>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
@@ -1415,8 +3945,8 @@
       <c r="A26" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="B26" s="9"/>
-      <c r="C26" s="8"/>
+      <c r="B26" s="17"/>
+      <c r="C26" s="18"/>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
@@ -1425,10 +3955,10 @@
       <c r="J26" s="1"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A27" s="9" t="s">
+      <c r="A27" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="B27" s="8"/>
+      <c r="B27" s="18"/>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
@@ -1438,13 +3968,13 @@
       <c r="J27" s="1"/>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A28" s="10" t="s">
+      <c r="A28" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="B28" s="8"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="8"/>
+      <c r="B28" s="18"/>
+      <c r="C28" s="18"/>
+      <c r="D28" s="18"/>
+      <c r="E28" s="18"/>
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
@@ -1452,10 +3982,10 @@
       <c r="J28" s="1"/>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A29" s="9" t="s">
+      <c r="A29" s="17" t="s">
         <v>76</v>
       </c>
-      <c r="B29" s="8"/>
+      <c r="B29" s="18"/>
       <c r="C29" s="1"/>
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
@@ -1465,12 +3995,12 @@
       <c r="J29" s="1"/>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A30" s="9" t="s">
+      <c r="A30" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="B30" s="8"/>
-      <c r="C30" s="8"/>
-      <c r="D30" s="8"/>
+      <c r="B30" s="18"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="18"/>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
@@ -1479,10 +4009,10 @@
       <c r="J30" s="1"/>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A31" s="9" t="s">
+      <c r="A31" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="B31" s="8"/>
+      <c r="B31" s="18"/>
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
@@ -1492,12 +4022,12 @@
       <c r="J31" s="1"/>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A32" s="9" t="s">
+      <c r="A32" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="B32" s="8"/>
-      <c r="C32" s="8"/>
-      <c r="D32" s="8"/>
+      <c r="B32" s="18"/>
+      <c r="C32" s="18"/>
+      <c r="D32" s="18"/>
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
       <c r="G32" s="1"/>
@@ -1506,10 +4036,10 @@
       <c r="J32" s="1"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A33" s="9" t="s">
+      <c r="A33" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="B33" s="8"/>
+      <c r="B33" s="18"/>
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
       <c r="E33" s="1"/>
@@ -1520,12 +4050,12 @@
       <c r="J33" s="1"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A34" s="9" t="s">
+      <c r="A34" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="B34" s="8"/>
-      <c r="C34" s="8"/>
-      <c r="D34" s="8"/>
+      <c r="B34" s="18"/>
+      <c r="C34" s="18"/>
+      <c r="D34" s="18"/>
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
       <c r="G34" s="1"/>
@@ -1534,10 +4064,10 @@
       <c r="J34" s="1"/>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A35" s="9" t="s">
+      <c r="A35" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="B35" s="8"/>
+      <c r="B35" s="18"/>
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
       <c r="E35" s="1"/>
@@ -1548,12 +4078,12 @@
       <c r="J35" s="1"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A36" s="9" t="s">
+      <c r="A36" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="B36" s="8"/>
-      <c r="C36" s="8"/>
-      <c r="D36" s="8"/>
+      <c r="B36" s="18"/>
+      <c r="C36" s="18"/>
+      <c r="D36" s="18"/>
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
       <c r="G36" s="1"/>
@@ -1562,10 +4092,10 @@
       <c r="J36" s="1"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A37" s="9" t="s">
+      <c r="A37" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="B37" s="8"/>
+      <c r="B37" s="18"/>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" s="1"/>
@@ -1627,21 +4157,6 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="A34:D34"/>
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="A36:D36"/>
     <mergeCell ref="A37:B37"/>
@@ -1652,6 +4167,21 @@
     <mergeCell ref="A31:B31"/>
     <mergeCell ref="A32:D32"/>
     <mergeCell ref="A33:B33"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="B8:D8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: toi uu dem nguoi vao tiec khong bi rot, dang nhap van tay uu tien va QA tu dong cong bo sau 15s
</commit_message>
<xml_diff>
--- a/Team Building TCKT.xlsx
+++ b/Team Building TCKT.xlsx
@@ -8,22 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NHANDQ\Downloads\TeamBuilding\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A033379F-AF2E-4A91-B8CF-DED03A245CD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FEC3BBC-1557-4405-9C45-CD930C88CB47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6480" yWindow="4905" windowWidth="21600" windowHeight="11385" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Squizz" sheetId="3" r:id="rId1"/>
     <sheet name="Danh sách tham gia" sheetId="5" r:id="rId2"/>
-    <sheet name="Sheet2" sheetId="6" r:id="rId3"/>
-    <sheet name="Bộ Q&amp;A" sheetId="4" r:id="rId4"/>
+    <sheet name="Bộ Q&amp;A" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="181">
   <si>
     <t>BỘ 10 CÂU HỎI NHẬP TÊN CHO QUIZIZZ</t>
   </si>
@@ -561,105 +560,6 @@
   </si>
   <si>
     <t>Ngày tháng năm sinh</t>
-  </si>
-  <si>
-    <t>13/12/1994</t>
-  </si>
-  <si>
-    <t>13/11/2002</t>
-  </si>
-  <si>
-    <t>19/03/2002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26/06/1992 </t>
-  </si>
-  <si>
-    <t>18/04/2000</t>
-  </si>
-  <si>
-    <t>16/12/2003</t>
-  </si>
-  <si>
-    <t>23/12/1990</t>
-  </si>
-  <si>
-    <t>25/6/1991</t>
-  </si>
-  <si>
-    <t>20/12/1981</t>
-  </si>
-  <si>
-    <t>22/4/1987</t>
-  </si>
-  <si>
-    <t>14/10/2001</t>
-  </si>
-  <si>
-    <t>17/05/1990</t>
-  </si>
-  <si>
-    <t>23/12/1992</t>
-  </si>
-  <si>
-    <t>22/11/1999</t>
-  </si>
-  <si>
-    <t>27/06/2002</t>
-  </si>
-  <si>
-    <t>26/07/2002</t>
-  </si>
-  <si>
-    <t>27/07/2003</t>
-  </si>
-  <si>
-    <t>31/10/2002</t>
-  </si>
-  <si>
-    <t>20/06/2004</t>
-  </si>
-  <si>
-    <t>14/01/1992</t>
-  </si>
-  <si>
-    <t>02/08/1994</t>
-  </si>
-  <si>
-    <t>28/12/2002</t>
-  </si>
-  <si>
-    <t>02/05/2001</t>
-  </si>
-  <si>
-    <t>15/05/1996</t>
-  </si>
-  <si>
-    <t>13/10/2003</t>
-  </si>
-  <si>
-    <t>23/03/2004</t>
-  </si>
-  <si>
-    <t>30/04/1996</t>
-  </si>
-  <si>
-    <t>27/12/1983</t>
-  </si>
-  <si>
-    <t>29/03/2003</t>
-  </si>
-  <si>
-    <t>19/02/2003</t>
-  </si>
-  <si>
-    <t>21/09/2005</t>
-  </si>
-  <si>
-    <t>18/06/2025</t>
-  </si>
-  <si>
-    <t>29/09/2004</t>
   </si>
   <si>
     <t>VIP</t>
@@ -675,7 +575,7 @@
   <numFmts count="1">
     <numFmt numFmtId="168" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -770,24 +670,6 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FFFF0000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -803,7 +685,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -856,161 +738,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="hair">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="hair">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="hair">
-        <color indexed="64"/>
-      </top>
-      <bottom style="hair">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="hair">
-        <color indexed="64"/>
-      </top>
-      <bottom style="hair">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="hair">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="hair">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="hair">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="hair">
-        <color indexed="64"/>
-      </top>
-      <bottom style="hair">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1068,74 +802,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="14" fontId="11" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="11" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="11" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="11" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="13" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="11" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="11" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="15" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="11" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="11" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="11" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1729,7 +1395,7 @@
     <col min="2" max="2" width="23" style="29" customWidth="1"/>
     <col min="3" max="3" width="25.7109375" customWidth="1"/>
     <col min="4" max="4" width="16.42578125" customWidth="1"/>
-    <col min="5" max="5" width="26.140625" style="55" customWidth="1"/>
+    <col min="5" max="5" width="26.140625" style="31" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1745,7 +1411,7 @@
       <c r="D1" s="22" t="s">
         <v>177</v>
       </c>
-      <c r="E1" s="54" t="s">
+      <c r="E1" s="30" t="s">
         <v>178</v>
       </c>
     </row>
@@ -1762,7 +1428,7 @@
       <c r="D2" s="24">
         <v>6</v>
       </c>
-      <c r="E2" s="55">
+      <c r="E2" s="31">
         <v>33873</v>
       </c>
     </row>
@@ -1779,7 +1445,7 @@
       <c r="D3" s="25">
         <v>1770</v>
       </c>
-      <c r="E3" s="55">
+      <c r="E3" s="31">
         <v>33438</v>
       </c>
     </row>
@@ -1796,7 +1462,7 @@
       <c r="D4" s="25">
         <v>8</v>
       </c>
-      <c r="E4" s="55">
+      <c r="E4" s="31">
         <v>34857</v>
       </c>
     </row>
@@ -1813,7 +1479,7 @@
       <c r="D5" s="25">
         <v>2539</v>
       </c>
-      <c r="E5" s="55">
+      <c r="E5" s="31">
         <v>32742</v>
       </c>
     </row>
@@ -1830,7 +1496,7 @@
       <c r="D6" s="25">
         <v>381</v>
       </c>
-      <c r="E6" s="55">
+      <c r="E6" s="31">
         <v>35183</v>
       </c>
     </row>
@@ -1847,7 +1513,7 @@
       <c r="D7" s="25">
         <v>3765</v>
       </c>
-      <c r="E7" s="55">
+      <c r="E7" s="31">
         <v>33775</v>
       </c>
     </row>
@@ -1864,7 +1530,7 @@
       <c r="D8" s="25">
         <v>2310</v>
       </c>
-      <c r="E8" s="54">
+      <c r="E8" s="30">
         <v>34681</v>
       </c>
     </row>
@@ -1881,7 +1547,7 @@
       <c r="D9" s="25">
         <v>3761</v>
       </c>
-      <c r="E9" s="55">
+      <c r="E9" s="31">
         <v>36483</v>
       </c>
     </row>
@@ -1898,7 +1564,7 @@
       <c r="D10" s="25">
         <v>1437</v>
       </c>
-      <c r="E10" s="55">
+      <c r="E10" s="31">
         <v>36122</v>
       </c>
     </row>
@@ -1915,7 +1581,7 @@
       <c r="D11" s="25">
         <v>1717</v>
       </c>
-      <c r="E11" s="55">
+      <c r="E11" s="31">
         <v>36171</v>
       </c>
     </row>
@@ -1932,7 +1598,7 @@
       <c r="D12" s="25">
         <v>2462</v>
       </c>
-      <c r="E12" s="55">
+      <c r="E12" s="31">
         <v>34230</v>
       </c>
     </row>
@@ -1949,7 +1615,7 @@
       <c r="D13" s="25">
         <v>2836</v>
       </c>
-      <c r="E13" s="55">
+      <c r="E13" s="31">
         <v>37046</v>
       </c>
     </row>
@@ -1966,7 +1632,7 @@
       <c r="D14" s="25">
         <v>3398</v>
       </c>
-      <c r="E14" s="55">
+      <c r="E14" s="31">
         <v>35769</v>
       </c>
     </row>
@@ -1983,7 +1649,7 @@
       <c r="D15" s="25">
         <v>4210</v>
       </c>
-      <c r="E15" s="55">
+      <c r="E15" s="31">
         <v>37723</v>
       </c>
     </row>
@@ -2000,7 +1666,7 @@
       <c r="D16" s="25">
         <v>4339</v>
       </c>
-      <c r="E16" s="55">
+      <c r="E16" s="31">
         <v>35675</v>
       </c>
     </row>
@@ -2017,7 +1683,7 @@
       <c r="D17" s="25">
         <v>4151</v>
       </c>
-      <c r="E17" s="55">
+      <c r="E17" s="31">
         <v>37334</v>
       </c>
     </row>
@@ -2034,7 +1700,7 @@
       <c r="D18" s="25">
         <v>5117</v>
       </c>
-      <c r="E18" s="55">
+      <c r="E18" s="31">
         <v>37324</v>
       </c>
     </row>
@@ -2051,7 +1717,7 @@
       <c r="D19" s="25">
         <v>5679</v>
       </c>
-      <c r="E19" s="55">
+      <c r="E19" s="31">
         <v>33781</v>
       </c>
     </row>
@@ -2068,7 +1734,7 @@
       <c r="D20" s="25">
         <v>5788</v>
       </c>
-      <c r="E20" s="55">
+      <c r="E20" s="31">
         <v>38025</v>
       </c>
     </row>
@@ -2085,7 +1751,7 @@
       <c r="D21" s="25">
         <v>5823</v>
       </c>
-      <c r="E21" s="55">
+      <c r="E21" s="31">
         <v>36903</v>
       </c>
     </row>
@@ -2102,7 +1768,7 @@
       <c r="D22" s="25">
         <v>3159</v>
       </c>
-      <c r="E22" s="55">
+      <c r="E22" s="31">
         <v>34548</v>
       </c>
     </row>
@@ -2119,7 +1785,7 @@
       <c r="D23" s="25">
         <v>3628</v>
       </c>
-      <c r="E23" s="55">
+      <c r="E23" s="31">
         <v>36565</v>
       </c>
     </row>
@@ -2136,7 +1802,7 @@
       <c r="D24" s="25">
         <v>4257</v>
       </c>
-      <c r="E24" s="55">
+      <c r="E24" s="31">
         <v>33010</v>
       </c>
     </row>
@@ -2153,7 +1819,7 @@
       <c r="D25" s="25">
         <v>6040</v>
       </c>
-      <c r="E25" s="55">
+      <c r="E25" s="31">
         <v>36486</v>
       </c>
     </row>
@@ -2170,7 +1836,7 @@
       <c r="D26" s="25">
         <v>4049</v>
       </c>
-      <c r="E26" s="55">
+      <c r="E26" s="31">
         <v>37434</v>
       </c>
     </row>
@@ -2187,7 +1853,7 @@
       <c r="D27" s="25">
         <v>4048</v>
       </c>
-      <c r="E27" s="55">
+      <c r="E27" s="31">
         <v>37463</v>
       </c>
     </row>
@@ -2204,7 +1870,7 @@
       <c r="D28" s="25">
         <v>4330</v>
       </c>
-      <c r="E28" s="55">
+      <c r="E28" s="31">
         <v>37829</v>
       </c>
     </row>
@@ -2221,7 +1887,7 @@
       <c r="D29" s="25">
         <v>4340</v>
       </c>
-      <c r="E29" s="55">
+      <c r="E29" s="31">
         <v>37560</v>
       </c>
     </row>
@@ -2238,7 +1904,7 @@
       <c r="D30" s="25">
         <v>4391</v>
       </c>
-      <c r="E30" s="55">
+      <c r="E30" s="31">
         <v>37927</v>
       </c>
     </row>
@@ -2255,7 +1921,7 @@
       <c r="D31" s="25">
         <v>5381</v>
       </c>
-      <c r="E31" s="55">
+      <c r="E31" s="31">
         <v>38158</v>
       </c>
     </row>
@@ -2272,7 +1938,7 @@
       <c r="D32" s="25">
         <v>5821</v>
       </c>
-      <c r="E32" s="55">
+      <c r="E32" s="31">
         <v>38330</v>
       </c>
     </row>
@@ -2289,7 +1955,7 @@
       <c r="D33" s="25">
         <v>6038</v>
       </c>
-      <c r="E33" s="54">
+      <c r="E33" s="30">
         <v>37983</v>
       </c>
     </row>
@@ -2306,7 +1972,7 @@
       <c r="D34" s="25">
         <v>2503</v>
       </c>
-      <c r="E34" s="55">
+      <c r="E34" s="31">
         <v>33617</v>
       </c>
     </row>
@@ -2323,7 +1989,7 @@
       <c r="D35" s="25">
         <v>4159</v>
       </c>
-      <c r="E35" s="55">
+      <c r="E35" s="31">
         <v>37013</v>
       </c>
     </row>
@@ -2340,7 +2006,7 @@
       <c r="D36" s="25">
         <v>4404</v>
       </c>
-      <c r="E36" s="55">
+      <c r="E36" s="31">
         <v>35200</v>
       </c>
     </row>
@@ -2357,7 +2023,7 @@
       <c r="D37" s="25">
         <v>4846</v>
       </c>
-      <c r="E37" s="55">
+      <c r="E37" s="31">
         <v>37907</v>
       </c>
     </row>
@@ -2374,7 +2040,7 @@
       <c r="D38" s="25">
         <v>2971</v>
       </c>
-      <c r="E38" s="55">
+      <c r="E38" s="31">
         <v>36490</v>
       </c>
     </row>
@@ -2391,7 +2057,7 @@
       <c r="D39" s="25">
         <v>2877</v>
       </c>
-      <c r="E39" s="55">
+      <c r="E39" s="31">
         <v>36903</v>
       </c>
     </row>
@@ -2408,7 +2074,7 @@
       <c r="D40" s="25">
         <v>4565</v>
       </c>
-      <c r="E40" s="55">
+      <c r="E40" s="31">
         <v>33516</v>
       </c>
     </row>
@@ -2425,7 +2091,7 @@
       <c r="D41" s="25">
         <v>886</v>
       </c>
-      <c r="E41" s="55">
+      <c r="E41" s="31">
         <v>34777</v>
       </c>
     </row>
@@ -2442,7 +2108,7 @@
       <c r="D42" s="25">
         <v>3958</v>
       </c>
-      <c r="E42" s="55">
+      <c r="E42" s="31">
         <v>37505</v>
       </c>
     </row>
@@ -2459,7 +2125,7 @@
       <c r="D43" s="25">
         <v>2144</v>
       </c>
-      <c r="E43" s="55">
+      <c r="E43" s="31">
         <v>36938</v>
       </c>
     </row>
@@ -2476,7 +2142,7 @@
       <c r="D44" s="25">
         <v>3379</v>
       </c>
-      <c r="E44" s="55">
+      <c r="E44" s="31">
         <v>34462</v>
       </c>
     </row>
@@ -2493,7 +2159,7 @@
       <c r="D45" s="25">
         <v>2200</v>
       </c>
-      <c r="E45" s="55">
+      <c r="E45" s="31">
         <v>33414</v>
       </c>
     </row>
@@ -2505,12 +2171,12 @@
         <v>140</v>
       </c>
       <c r="C46" s="28" t="s">
-        <v>212</v>
+        <v>179</v>
       </c>
       <c r="D46" s="21">
         <v>641</v>
       </c>
-      <c r="E46" s="55" t="e">
+      <c r="E46" s="31" t="e">
         <v>#N/A</v>
       </c>
     </row>
@@ -2527,8 +2193,8 @@
       <c r="D47" s="25">
         <v>6248</v>
       </c>
-      <c r="E47" s="54" t="s">
-        <v>213</v>
+      <c r="E47" s="30" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -2544,7 +2210,7 @@
       <c r="D48" s="25">
         <v>5791</v>
       </c>
-      <c r="E48" s="54">
+      <c r="E48" s="30">
         <v>38160</v>
       </c>
     </row>
@@ -2554,1016 +2220,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4846012-1C8E-45A4-8F94-FFA376830FDA}">
-  <dimension ref="A1:B131"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="13.42578125" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="31" t="s">
-        <v>177</v>
-      </c>
-      <c r="B1" s="47" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="33">
-        <v>6</v>
-      </c>
-      <c r="B2" s="48">
-        <v>33873</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="36">
-        <v>1770</v>
-      </c>
-      <c r="B3" s="49">
-        <v>33438</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="35">
-        <v>8</v>
-      </c>
-      <c r="B4" s="49">
-        <v>34886</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="37">
-        <v>2539</v>
-      </c>
-      <c r="B5" s="49">
-        <v>32742</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="36">
-        <v>381</v>
-      </c>
-      <c r="B6" s="49">
-        <v>35183</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="37">
-        <v>3765</v>
-      </c>
-      <c r="B7" s="49">
-        <v>33775</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="37">
-        <v>2310</v>
-      </c>
-      <c r="B8" s="49" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="37">
-        <v>3761</v>
-      </c>
-      <c r="B9" s="49">
-        <v>36483</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="36">
-        <v>1236</v>
-      </c>
-      <c r="B10" s="49">
-        <v>33332</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="36">
-        <v>1437</v>
-      </c>
-      <c r="B11" s="49">
-        <v>36122</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="35">
-        <v>1717</v>
-      </c>
-      <c r="B12" s="49">
-        <v>36465</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="37">
-        <v>2462</v>
-      </c>
-      <c r="B13" s="49">
-        <v>34230</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="36">
-        <v>2836</v>
-      </c>
-      <c r="B14" s="49">
-        <v>36987</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="35">
-        <v>3398</v>
-      </c>
-      <c r="B15" s="49">
-        <v>35562</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="37">
-        <v>4210</v>
-      </c>
-      <c r="B16" s="49">
-        <v>37959</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="37">
-        <v>4663</v>
-      </c>
-      <c r="B17" s="49" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="37">
-        <v>4339</v>
-      </c>
-      <c r="B18" s="49">
-        <v>35470</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="37">
-        <v>4151</v>
-      </c>
-      <c r="B19" s="49" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="37">
-        <v>5117</v>
-      </c>
-      <c r="B20" s="49">
-        <v>37502</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="37">
-        <v>5679</v>
-      </c>
-      <c r="B21" s="49" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="37">
-        <v>5426</v>
-      </c>
-      <c r="B22" s="49" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="37">
-        <v>5747</v>
-      </c>
-      <c r="B23" s="49" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="37">
-        <v>5788</v>
-      </c>
-      <c r="B24" s="49">
-        <v>38201</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="37">
-        <v>5823</v>
-      </c>
-      <c r="B25" s="49">
-        <v>37226</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="32"/>
-      <c r="B26" s="50"/>
-    </row>
-    <row r="27" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="38">
-        <v>1862</v>
-      </c>
-      <c r="B27" s="44" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="36">
-        <v>2973</v>
-      </c>
-      <c r="B28" s="43" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A29" s="37">
-        <v>3326</v>
-      </c>
-      <c r="B29" s="43">
-        <v>31626</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="37">
-        <v>3268</v>
-      </c>
-      <c r="B30" s="43" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A31" s="37">
-        <v>4013</v>
-      </c>
-      <c r="B31" s="43" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A32" s="37">
-        <v>3306</v>
-      </c>
-      <c r="B32" s="43" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A33" s="37">
-        <v>3628</v>
-      </c>
-      <c r="B33" s="43">
-        <v>36771</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A34" s="37">
-        <v>4257</v>
-      </c>
-      <c r="B34" s="43" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A35" s="37">
-        <v>5789</v>
-      </c>
-      <c r="B35" s="43">
-        <v>30691</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A36" s="37">
-        <v>5328</v>
-      </c>
-      <c r="B36" s="43" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A37" s="38">
-        <v>6040</v>
-      </c>
-      <c r="B37" s="51" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A38" s="32"/>
-      <c r="B38" s="50"/>
-    </row>
-    <row r="39" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A39" s="37">
-        <v>4049</v>
-      </c>
-      <c r="B39" s="45" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A40" s="37">
-        <v>4048</v>
-      </c>
-      <c r="B40" s="43" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A41" s="37">
-        <v>4047</v>
-      </c>
-      <c r="B41" s="43">
-        <v>37961</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A42" s="37">
-        <v>4330</v>
-      </c>
-      <c r="B42" s="43" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A43" s="37">
-        <v>4340</v>
-      </c>
-      <c r="B43" s="43" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A44" s="37">
-        <v>4391</v>
-      </c>
-      <c r="B44" s="43">
-        <v>37663</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A45" s="37">
-        <v>5381</v>
-      </c>
-      <c r="B45" s="43" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A46" s="37">
-        <v>5675</v>
-      </c>
-      <c r="B46" s="43">
-        <v>36536</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A47" s="37">
-        <v>5821</v>
-      </c>
-      <c r="B47" s="43">
-        <v>38242</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48" s="30"/>
-      <c r="B48" s="42"/>
-    </row>
-    <row r="49" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A49" s="37"/>
-      <c r="B49" s="49"/>
-    </row>
-    <row r="50" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A50" s="37"/>
-      <c r="B50" s="49"/>
-    </row>
-    <row r="51" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A51" s="40"/>
-      <c r="B51" s="50"/>
-    </row>
-    <row r="52" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A52" s="34">
-        <v>2503</v>
-      </c>
-      <c r="B52" s="52" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A53" s="37">
-        <v>3159</v>
-      </c>
-      <c r="B53" s="52" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A54" s="37">
-        <v>3269</v>
-      </c>
-      <c r="B54" s="49" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A55" s="37">
-        <v>4159</v>
-      </c>
-      <c r="B55" s="52" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A56" s="37">
-        <v>4404</v>
-      </c>
-      <c r="B56" s="52" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A57" s="37">
-        <v>4846</v>
-      </c>
-      <c r="B57" s="52" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A58" s="37">
-        <v>6014</v>
-      </c>
-      <c r="B58" s="52" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A59" s="37"/>
-      <c r="B59" s="52"/>
-    </row>
-    <row r="60" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A60" s="37"/>
-      <c r="B60" s="52"/>
-    </row>
-    <row r="61" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A61" s="37"/>
-      <c r="B61" s="52"/>
-    </row>
-    <row r="62" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A62" s="40"/>
-      <c r="B62" s="50"/>
-    </row>
-    <row r="63" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A63" s="33">
-        <v>1790</v>
-      </c>
-      <c r="B63" s="48">
-        <v>31292</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A64" s="36">
-        <v>2077</v>
-      </c>
-      <c r="B64" s="49">
-        <v>36652</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A65" s="37">
-        <v>2200</v>
-      </c>
-      <c r="B65" s="49">
-        <v>33414</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A66" s="35">
-        <v>2209</v>
-      </c>
-      <c r="B66" s="49">
-        <v>30572</v>
-      </c>
-    </row>
-    <row r="67" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A67" s="36">
-        <v>2560</v>
-      </c>
-      <c r="B67" s="49">
-        <v>37033</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A68" s="35">
-        <v>2569</v>
-      </c>
-      <c r="B68" s="49">
-        <v>36919</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A69" s="36">
-        <v>2622</v>
-      </c>
-      <c r="B69" s="49">
-        <v>37108</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A70" s="36">
-        <v>2680</v>
-      </c>
-      <c r="B70" s="49">
-        <v>37178</v>
-      </c>
-    </row>
-    <row r="71" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A71" s="36">
-        <v>2805</v>
-      </c>
-      <c r="B71" s="49">
-        <v>36541</v>
-      </c>
-    </row>
-    <row r="72" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A72" s="36">
-        <v>3041</v>
-      </c>
-      <c r="B72" s="49">
-        <v>35692</v>
-      </c>
-    </row>
-    <row r="73" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A73" s="37">
-        <v>2668</v>
-      </c>
-      <c r="B73" s="49">
-        <v>35202</v>
-      </c>
-    </row>
-    <row r="74" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A74" s="35">
-        <v>1811</v>
-      </c>
-      <c r="B74" s="49">
-        <v>35395</v>
-      </c>
-    </row>
-    <row r="75" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A75" s="37">
-        <v>2143</v>
-      </c>
-      <c r="B75" s="49">
-        <v>36018</v>
-      </c>
-    </row>
-    <row r="76" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A76" s="35">
-        <v>886</v>
-      </c>
-      <c r="B76" s="49">
-        <v>34777</v>
-      </c>
-    </row>
-    <row r="77" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A77" s="35">
-        <v>2563</v>
-      </c>
-      <c r="B77" s="49">
-        <v>36264</v>
-      </c>
-    </row>
-    <row r="78" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A78" s="35">
-        <v>2293</v>
-      </c>
-      <c r="B78" s="49">
-        <v>34924</v>
-      </c>
-    </row>
-    <row r="79" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A79" s="35">
-        <v>2494</v>
-      </c>
-      <c r="B79" s="49">
-        <v>36174</v>
-      </c>
-    </row>
-    <row r="80" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A80" s="35">
-        <v>2971</v>
-      </c>
-      <c r="B80" s="49">
-        <v>36490</v>
-      </c>
-    </row>
-    <row r="81" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A81" s="35">
-        <v>2877</v>
-      </c>
-      <c r="B81" s="49">
-        <v>37226</v>
-      </c>
-    </row>
-    <row r="82" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A82" s="35">
-        <v>3363</v>
-      </c>
-      <c r="B82" s="49">
-        <v>36854</v>
-      </c>
-    </row>
-    <row r="83" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A83" s="35">
-        <v>3426</v>
-      </c>
-      <c r="B83" s="49">
-        <v>37569</v>
-      </c>
-    </row>
-    <row r="84" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A84" s="35">
-        <v>3476</v>
-      </c>
-      <c r="B84" s="49">
-        <v>36571</v>
-      </c>
-    </row>
-    <row r="85" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A85" s="35">
-        <v>3474</v>
-      </c>
-      <c r="B85" s="49">
-        <v>36950</v>
-      </c>
-    </row>
-    <row r="86" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A86" s="35">
-        <v>3379</v>
-      </c>
-      <c r="B86" s="49">
-        <v>34551</v>
-      </c>
-    </row>
-    <row r="87" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A87" s="35">
-        <v>670</v>
-      </c>
-      <c r="B87" s="49"/>
-    </row>
-    <row r="88" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A88" s="35">
-        <v>850</v>
-      </c>
-      <c r="B88" s="49">
-        <v>30187</v>
-      </c>
-    </row>
-    <row r="89" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A89" s="35">
-        <v>2144</v>
-      </c>
-      <c r="B89" s="49">
-        <v>36938</v>
-      </c>
-    </row>
-    <row r="90" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A90" s="39">
-        <v>3958</v>
-      </c>
-      <c r="B90" s="49">
-        <v>37416</v>
-      </c>
-    </row>
-    <row r="91" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A91" s="32"/>
-      <c r="B91" s="50"/>
-    </row>
-    <row r="92" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A92" s="35">
-        <v>1779</v>
-      </c>
-      <c r="B92" s="49">
-        <v>29064</v>
-      </c>
-    </row>
-    <row r="93" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A93" s="32"/>
-      <c r="B93" s="50"/>
-    </row>
-    <row r="94" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A94" s="41">
-        <v>1179</v>
-      </c>
-      <c r="B94" s="49">
-        <v>32435</v>
-      </c>
-    </row>
-    <row r="95" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A95" s="35">
-        <v>252</v>
-      </c>
-      <c r="B95" s="49">
-        <v>32396</v>
-      </c>
-    </row>
-    <row r="96" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A96" s="35">
-        <v>3648</v>
-      </c>
-      <c r="B96" s="49">
-        <v>32642</v>
-      </c>
-    </row>
-    <row r="97" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A97" s="35">
-        <v>3681</v>
-      </c>
-      <c r="B97" s="52">
-        <v>33311</v>
-      </c>
-    </row>
-    <row r="98" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A98" s="35">
-        <v>3535</v>
-      </c>
-      <c r="B98" s="49">
-        <v>34101</v>
-      </c>
-    </row>
-    <row r="99" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A99" s="36">
-        <v>1124</v>
-      </c>
-      <c r="B99" s="49">
-        <v>33345</v>
-      </c>
-    </row>
-    <row r="100" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A100" s="37">
-        <v>3488</v>
-      </c>
-      <c r="B100" s="49">
-        <v>34357</v>
-      </c>
-    </row>
-    <row r="101" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A101" s="35">
-        <v>2054</v>
-      </c>
-      <c r="B101" s="49"/>
-    </row>
-    <row r="102" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A102" s="37">
-        <v>3946</v>
-      </c>
-      <c r="B102" s="49">
-        <v>36996</v>
-      </c>
-    </row>
-    <row r="103" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A103" s="37">
-        <v>3943</v>
-      </c>
-      <c r="B103" s="49">
-        <v>37322</v>
-      </c>
-    </row>
-    <row r="104" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A104" s="37">
-        <v>3936</v>
-      </c>
-      <c r="B104" s="49">
-        <v>37032</v>
-      </c>
-    </row>
-    <row r="105" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A105" s="37">
-        <v>3937</v>
-      </c>
-      <c r="B105" s="49">
-        <v>36164</v>
-      </c>
-    </row>
-    <row r="106" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A106" s="37">
-        <v>2954</v>
-      </c>
-      <c r="B106" s="49">
-        <v>34138</v>
-      </c>
-    </row>
-    <row r="107" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A107" s="37">
-        <v>3588</v>
-      </c>
-      <c r="B107" s="49">
-        <v>36638</v>
-      </c>
-    </row>
-    <row r="108" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A108" s="37">
-        <v>4182</v>
-      </c>
-      <c r="B108" s="49">
-        <v>37322</v>
-      </c>
-    </row>
-    <row r="109" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A109" s="37">
-        <v>3511</v>
-      </c>
-      <c r="B109" s="49">
-        <v>35386</v>
-      </c>
-    </row>
-    <row r="110" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A110" s="37">
-        <v>3870</v>
-      </c>
-      <c r="B110" s="49">
-        <v>36912</v>
-      </c>
-    </row>
-    <row r="111" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A111" s="37">
-        <v>4186</v>
-      </c>
-      <c r="B111" s="49">
-        <v>35491</v>
-      </c>
-    </row>
-    <row r="112" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A112" s="37">
-        <v>4502</v>
-      </c>
-      <c r="B112" s="49" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="113" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A113" s="37">
-        <v>4495</v>
-      </c>
-      <c r="B113" s="49" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="114" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A114" s="37">
-        <v>3910</v>
-      </c>
-      <c r="B114" s="49">
-        <v>35424</v>
-      </c>
-    </row>
-    <row r="115" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A115" s="37">
-        <v>4352</v>
-      </c>
-      <c r="B115" s="49">
-        <v>37349</v>
-      </c>
-    </row>
-    <row r="116" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A116" s="37">
-        <v>2638</v>
-      </c>
-      <c r="B116" s="53">
-        <v>33989</v>
-      </c>
-    </row>
-    <row r="117" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A117" s="37">
-        <v>4888</v>
-      </c>
-      <c r="B117" s="49">
-        <v>36590</v>
-      </c>
-    </row>
-    <row r="118" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A118" s="37">
-        <v>4320</v>
-      </c>
-      <c r="B118" s="49">
-        <v>37838</v>
-      </c>
-    </row>
-    <row r="119" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A119" s="37">
-        <v>4887</v>
-      </c>
-      <c r="B119" s="49">
-        <v>37804</v>
-      </c>
-    </row>
-    <row r="120" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A120" s="37">
-        <v>4422</v>
-      </c>
-      <c r="B120" s="49">
-        <v>37692</v>
-      </c>
-    </row>
-    <row r="121" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A121" s="37">
-        <v>4296</v>
-      </c>
-      <c r="B121" s="49" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="122" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A122" s="37">
-        <v>4351</v>
-      </c>
-      <c r="B122" s="49">
-        <v>37690</v>
-      </c>
-    </row>
-    <row r="123" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A123" s="37">
-        <v>4295</v>
-      </c>
-      <c r="B123" s="49" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="124" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A124" s="37">
-        <v>5229</v>
-      </c>
-      <c r="B124" s="49">
-        <v>32662</v>
-      </c>
-    </row>
-    <row r="125" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A125" s="37">
-        <v>5170</v>
-      </c>
-      <c r="B125" s="49">
-        <v>37149</v>
-      </c>
-    </row>
-    <row r="126" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A126" s="37">
-        <v>4782</v>
-      </c>
-      <c r="B126" s="49" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="127" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A127" s="37">
-        <v>4680</v>
-      </c>
-      <c r="B127" s="49" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="128" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A128" s="37">
-        <v>5742</v>
-      </c>
-      <c r="B128" s="49">
-        <v>37811</v>
-      </c>
-    </row>
-    <row r="129" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A129" s="37">
-        <v>4358</v>
-      </c>
-      <c r="B129" s="49">
-        <v>37662</v>
-      </c>
-    </row>
-    <row r="130" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A130" s="37">
-        <v>5632</v>
-      </c>
-      <c r="B130" s="52">
-        <v>36258</v>
-      </c>
-    </row>
-    <row r="131" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A131" s="37">
-        <v>5631</v>
-      </c>
-      <c r="B131" s="46" t="s">
-        <v>211</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>

</xml_diff>